<commit_message>
docs(qa): enhance test spreadsheets with beginner-friendly instructions
- Add dedicated Actions_Tests.xlsx with 13 sheets covering all 11 action types
- Extract Actions and Action Validation sheets from Activity_Tests.xlsx
- Enhance all test files with detailed step-by-step instructions
- Add bold headers to all sheets for better readability
- Include explicit UI element locations and expected results

Test coverage:
- Actions_Tests.xlsx: ~105 tests (Assign, Seize, Release, Delay, etc.)
- Activity_Tests.xlsx: 8 sheets (removed Actions sheets)
- Resource_Tests.xlsx: 8 sheets, 61 tests
- Duration_Editor_Tests.xlsx: 7 sheets, 70 tests
- Generator_Tests.xlsx, Entity_Tests.xlsx, Model_Tests.xlsx: enhanced
- Connector_Tests.xlsx: enhanced

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_qa/Resource_Tests.xlsx
+++ b/_qa/Resource_Tests.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="504">
   <si>
     <t>Test ID</t>
   </si>
@@ -892,6 +892,1266 @@
   </si>
   <si>
     <t>WARNING about potential overutilization</t>
+  </si>
+  <si>
+    <t>Navigate to Basic Settings tab</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Look at your diagram and find a Resource shape (displayed as a hexagon)
+3. Click on the Resource shape to select it
+4. The right panel should now show "Resource Editor"</t>
+  </si>
+  <si>
+    <t>1. Look at the tab bar at the top of the Resource Editor panel
+2. You should see 3 small icons in a row
+3. Find the gear icon (⚙️) - this is the FIRST icon on the left
+4. Click on the gear icon</t>
+  </si>
+  <si>
+    <t>1. The gear icon should now appear highlighted or selected
+2. The panel content below changes to show "Basic Settings"
+3. You should see a "Resource Name" text field near the top
+4. You should see a "Capacity" number field below the name</t>
+  </si>
+  <si>
+    <t>Navigate to Financial Settings tab</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. The Resource Editor panel is visible on the right
+3. You can see the 3 tab icons at the top of the panel</t>
+  </si>
+  <si>
+    <t>1. Look at the tab bar with 3 icons
+2. Find the dollar sign icon ($) - this is the SECOND/MIDDLE icon
+3. Click on the dollar sign icon</t>
+  </si>
+  <si>
+    <t>1. The dollar icon should now appear highlighted or selected
+2. The panel content changes to show "Financial Settings"
+3. You should see an "Enable Financial Tracking" checkbox
+4. Cost fields appear only when the checkbox is checked</t>
+  </si>
+  <si>
+    <t>1. Look at the tab bar with 3 icons
+2. Find the calendar/list icon - this is the THIRD icon on the right
+3. Click on the calendar/list icon</t>
+  </si>
+  <si>
+    <t>1. The States icon should now appear highlighted or selected
+2. The panel content changes to show the States editor
+3. You should see a list of resource states
+4. NOTE: This tab auto-saves - there is NO Save button</t>
+  </si>
+  <si>
+    <t>Verify all 3 tabs are visible</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. The Resource Editor panel is visible on the right</t>
+  </si>
+  <si>
+    <t>1. Look at the top of the Resource Editor panel
+2. Find the row of tab icons
+3. Count how many icons you see
+4. Identify each icon from left to right</t>
+  </si>
+  <si>
+    <t>1. You should see exactly 3 tab icons
+2. First icon (left): Gear icon (⚙️) = Basic Settings
+3. Second icon (middle): Dollar icon ($) = Financial Settings
+4. Third icon (right): Calendar/list icon = States</t>
+  </si>
+  <si>
+    <t>Tab tooltips display on hover</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. The Resource Editor panel is visible on the right
+3. You can see the 3 tab icons at the top</t>
+  </si>
+  <si>
+    <t>1. Move your mouse cursor over the first icon (gear)
+2. Hold it still for 1-2 seconds without clicking
+3. Repeat for the second icon (dollar sign)
+4. Repeat for the third icon (calendar/list)</t>
+  </si>
+  <si>
+    <t>1. When you hover over each icon, a small tooltip should appear
+2. The tooltip shows the name of that tab
+3. Gear icon tooltip: "Basic Settings" (or similar)
+4. Dollar icon tooltip: "Financial Settings" (or similar)
+5. Calendar icon tooltip: "States" (or similar)</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Click on a Resource shape (hexagon) in your diagram
+3. The Resource Editor panel appears on the right
+4. Click the gear icon (⚙️) to open Basic Settings tab
+5. You should see the "Resource Name" field near the top</t>
+  </si>
+  <si>
+    <t>1. Find the "Resource Name" text field at the top of the panel
+2. Click inside the text field - you'll see a blinking cursor
+3. Select all existing text (Ctrl+A or triple-click)
+4. Type a new name like "Test Worker"
+5. Press Tab or click somewhere outside the text field</t>
+  </si>
+  <si>
+    <t>1. The text field now shows your new name "Test Worker"
+2. Look at the bottom of the panel
+3. The "Save" button should now be BLUE and clickable (not grayed out)
+4. The "Cancel" button appears next to Save</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings tab is open (gear icon selected)
+3. You can see the "Capacity" field below the name field</t>
+  </si>
+  <si>
+    <t>1. Find the "Capacity" number field in the Basic Settings
+2. Click inside the Capacity field
+3. Clear the current value and type "5"
+4. Press Tab or click somewhere outside the field</t>
+  </si>
+  <si>
+    <t>1. The Capacity field now shows "5"
+2. The "Save" button at the bottom becomes BLUE and clickable
+3. This capacity means the resource can serve up to 5 activities at once</t>
+  </si>
+  <si>
+    <t>Minimum capacity enforced (zero rejected)</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings tab is open (gear icon selected)
+3. The Capacity field currently shows a valid number (like 1)</t>
+  </si>
+  <si>
+    <t>1. Find the "Capacity" number field
+2. Click inside the Capacity field
+3. Clear the current value and type "0"
+4. Press Tab or click somewhere outside the field</t>
+  </si>
+  <si>
+    <t>1. The Capacity field should NOT accept 0
+2. It should either revert to 1 automatically
+3. OR show an error/warning that capacity must be at least 1
+4. Resources must have at least 1 capacity to be useful</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings tab is open (gear icon selected)
+3. The Capacity field currently shows a valid number</t>
+  </si>
+  <si>
+    <t>1. Find the "Capacity" number field
+2. Click inside the Capacity field
+3. Clear the current value and type "-1" (negative one)
+4. Press Tab or click somewhere outside the field</t>
+  </si>
+  <si>
+    <t>1. The Capacity field should NOT accept negative numbers
+2. It should either revert to 1 automatically
+3. OR block the input entirely
+4. OR show an error that capacity must be positive</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings tab is open (gear icon selected)
+3. The Resource Name field shows a name</t>
+  </si>
+  <si>
+    <t>1. Find the "Resource Name" text field
+2. Click inside the text field
+3. Select all text and delete it completely (leave the field empty)
+4. Press Tab or click somewhere outside the field</t>
+  </si>
+  <si>
+    <t>1. The name field is now empty (blank)
+2. The application may either:
+   - Accept the empty name (field stays blank)
+   - Show a validation error or warning
+   - Revert to a default name
+3. Note what behavior you observe for the test result</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings tab is open (gear icon selected)
+3. The Resource Name field is visible</t>
+  </si>
+  <si>
+    <t>1. Find the "Resource Name" text field
+2. Click inside and select all existing text
+3. Type a name with special characters: "Test!@#$%Resource"
+4. Press Tab or click outside the field</t>
+  </si>
+  <si>
+    <t>1. The name field should accept special characters
+2. The field should display "Test!@#$%Resource"
+3. The Save button should become enabled
+4. Special characters are allowed in resource names</t>
+  </si>
+  <si>
+    <t>Very long name handling</t>
+  </si>
+  <si>
+    <t>1. Find the "Resource Name" text field
+2. Click inside and select all existing text
+3. Paste or type a very long name (500+ characters)
+   Example: repeat "LongResourceName" 35 times
+4. Press Tab or click outside the field</t>
+  </si>
+  <si>
+    <t>1. The application should handle the long name gracefully
+2. Either:
+   - Accept the full long name
+   - Truncate to a maximum length
+   - Show a validation warning about length
+3. The application should NOT crash or freeze</t>
+  </si>
+  <si>
+    <t>Capacity info tooltip displays</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings tab is open (gear icon selected)
+3. You can see the Capacity field with a small info icon (i or ?) next to it</t>
+  </si>
+  <si>
+    <t>1. Find the "Capacity" field label
+2. Look for a small info icon (i) or question mark (?) near the label
+3. Move your mouse cursor over this info icon
+4. Hold still for 1-2 seconds without clicking</t>
+  </si>
+  <si>
+    <t>1. A tooltip popup should appear near the info icon
+2. The tooltip explains what "Capacity" means:
+   - How many entities can use this resource simultaneously
+   - Example: Capacity of 3 means 3 activities can use the resource at once
+3. The tooltip disappears when you move your mouse away</t>
+  </si>
+  <si>
+    <t>Name info tooltip displays</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings tab is open (gear icon selected)
+3. You can see the Resource Name field with a small info icon next to it</t>
+  </si>
+  <si>
+    <t>1. Find the "Resource Name" field label
+2. Look for a small info icon (i) or question mark (?) near the label
+3. Move your mouse cursor over this info icon
+4. Hold still for 1-2 seconds without clicking</t>
+  </si>
+  <si>
+    <t>1. A tooltip popup should appear near the info icon
+2. The tooltip explains what the resource name is for:
+   - Identifying the resource in the model
+   - How it appears in simulation reports
+3. The tooltip disappears when you move your mouse away</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Click the dollar icon ($) in the tab bar to open Financial Settings
+3. You should see an "Enable Financial Tracking" checkbox at the top
+4. The checkbox is currently UNCHECKED</t>
+  </si>
+  <si>
+    <t>1. Look at the top of the Financial Settings panel
+2. Find the checkbox labeled "Enable Financial Tracking"
+3. Click directly on the checkbox (or the label text)
+4. The checkbox should now have a checkmark</t>
+  </si>
+  <si>
+    <t>1. The checkbox now shows a checkmark (is checked)
+2. New cost fields appear BELOW the checkbox:
+   - "Cost Per Seize"
+   - "Cost Per Hour Utilized"
+   - "Cost Per Hour Idle"
+3. Each cost field shows a default value (usually 0)
+4. The Save button becomes enabled</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Financial Settings tab is open (dollar icon selected)
+3. The "Enable Financial Tracking" checkbox is CHECKED
+4. Cost fields are visible below</t>
+  </si>
+  <si>
+    <t>1. Find the "Enable Financial Tracking" checkbox (currently checked)
+2. Click on the checkbox to UNCHECK it
+3. Watch the area below the checkbox</t>
+  </si>
+  <si>
+    <t>1. The checkbox is now UNCHECKED (no checkmark)
+2. All cost fields DISAPPEAR from view
+   - Cost Per Seize - HIDDEN
+   - Cost Per Hour Utilized - HIDDEN
+   - Cost Per Hour Idle - HIDDEN
+3. The panel looks simpler with just the checkbox visible
+4. The Save button becomes enabled to save this change</t>
+  </si>
+  <si>
+    <t>Edit Cost Per Seize field</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Financial Settings tab is open (dollar icon selected)
+3. "Enable Financial Tracking" is CHECKED
+4. Cost fields are visible</t>
+  </si>
+  <si>
+    <t>1. Find the "Cost Per Seize" field
+   (This is the cost incurred each time the resource is seized)
+2. Click inside the field
+3. Clear the current value and type "100"
+4. Press Tab or click outside the field</t>
+  </si>
+  <si>
+    <t>1. The Cost Per Seize field now shows "100"
+2. The Save button at the bottom becomes BLUE and clickable
+3. This means it costs $100 each time an activity seizes this resource</t>
+  </si>
+  <si>
+    <t>Edit Cost Per Hour Utilized field</t>
+  </si>
+  <si>
+    <t>1. Find the "Cost Per Hour Utilized" field
+   (This is the hourly cost when the resource is actively being used)
+2. Click inside the field
+3. Clear the current value and type "25"
+4. Press Tab or click outside the field</t>
+  </si>
+  <si>
+    <t>1. The Cost Per Hour Utilized field now shows "25"
+2. The Save button becomes enabled
+3. This means the resource costs $25 per hour while actively working</t>
+  </si>
+  <si>
+    <t>Edit Cost Per Hour Idle field</t>
+  </si>
+  <si>
+    <t>1. Find the "Cost Per Hour Idle" field
+   (This is the hourly cost when the resource is available but not being used)
+2. Click inside the field
+3. Clear the current value and type "5"
+4. Press Tab or click outside the field</t>
+  </si>
+  <si>
+    <t>1. The Cost Per Hour Idle field now shows "5"
+2. The Save button becomes enabled
+3. This means the resource costs $5 per hour while waiting/idle</t>
+  </si>
+  <si>
+    <t>Zero cost values accepted</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Financial Settings tab is open (dollar icon selected)
+3. "Enable Financial Tracking" is CHECKED
+4. Cost fields are visible with some non-zero values</t>
+  </si>
+  <si>
+    <t>1. Click inside the "Cost Per Seize" field and type "0"
+2. Click inside the "Cost Per Hour Utilized" field and type "0"
+3. Click inside the "Cost Per Hour Idle" field and type "0"
+4. Press Tab or click outside the fields</t>
+  </si>
+  <si>
+    <t>1. All three cost fields should accept the value 0
+2. The fields should display "0" (or "0.00")
+3. No error messages should appear
+4. The Save button should be enabled
+5. Zero costs are valid - some resources may have no cost</t>
+  </si>
+  <si>
+    <t>Decimal cost values accepted</t>
+  </si>
+  <si>
+    <t>1. Click inside any cost field (e.g., Cost Per Seize)
+2. Clear the current value
+3. Type a decimal value like "10.50"
+4. Press Tab or click outside the field</t>
+  </si>
+  <si>
+    <t>1. The cost field should accept the decimal value
+2. The field displays "10.50" (or similar decimal format)
+3. No error messages should appear
+4. The Save button should be enabled
+5. Decimal costs allow for precise financial tracking</t>
+  </si>
+  <si>
+    <t>Negative cost handling</t>
+  </si>
+  <si>
+    <t>1. Click inside any cost field (e.g., Cost Per Seize)
+2. Clear the current value
+3. Type a negative value like "-10"
+4. Press Tab or click outside the field</t>
+  </si>
+  <si>
+    <t>1. Check what the application does with negative costs
+2. Possible behaviors:
+   - Rejects the negative value (field resets to 0 or previous value)
+   - Accepts the negative value (could represent credits/refunds)
+   - Shows an error message
+3. Note the actual behavior for the test result</t>
+  </si>
+  <si>
+    <t>1. Find the "Cost Per Seize" field label
+2. Look for a small info icon (i) or question mark (?) near the label
+3. Move your mouse cursor over this info icon
+4. Hold still for 1-2 seconds without clicking</t>
+  </si>
+  <si>
+    <t>1. A tooltip popup should appear
+2. The tooltip explains what "Cost Per Seize" means:
+   - One-time cost incurred when an activity seizes the resource
+   - Charged once per seize operation
+3. The tooltip disappears when you move your mouse away</t>
+  </si>
+  <si>
+    <t>Cost Per Hour Utilized info tooltip</t>
+  </si>
+  <si>
+    <t>1. Find the "Cost Per Hour Utilized" field label
+2. Look for a small info icon (i) or question mark (?) near the label
+3. Move your mouse cursor over this info icon
+4. Hold still for 1-2 seconds without clicking</t>
+  </si>
+  <si>
+    <t>1. A tooltip popup should appear
+2. The tooltip explains what "Cost Per Hour Utilized" means:
+   - Hourly cost while the resource is actively being used
+   - Accumulates over time the resource is working
+3. The tooltip disappears when you move your mouse away</t>
+  </si>
+  <si>
+    <t>Cost Per Hour Idle info tooltip</t>
+  </si>
+  <si>
+    <t>1. Find the "Cost Per Hour Idle" field label
+2. Look for a small info icon (i) or question mark (?) near the label
+3. Move your mouse cursor over this info icon
+4. Hold still for 1-2 seconds without clicking</t>
+  </si>
+  <si>
+    <t>1. A tooltip popup should appear
+2. The tooltip explains what "Cost Per Hour Idle" means:
+   - Hourly cost while the resource is available but not in use
+   - Represents standby or waiting costs
+3. The tooltip disappears when you move your mouse away</t>
+  </si>
+  <si>
+    <t>Large cost values handling</t>
+  </si>
+  <si>
+    <t>1. Click inside any cost field (e.g., Cost Per Hour Utilized)
+2. Clear the current value
+3. Type a large value like "999999.99"
+4. Press Tab or click outside the field</t>
+  </si>
+  <si>
+    <t>1. The cost field should handle the large value gracefully
+2. The field should display the value (possibly formatted)
+3. No error messages should appear
+4. The application should NOT crash or freeze
+5. The Save button should be enabled</t>
+  </si>
+  <si>
+    <t>Stepper arrows increment cost</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Financial Settings tab is open (dollar icon selected)
+3. "Enable Financial Tracking" is CHECKED
+4. Cost fields are visible
+5. Look for small up/down arrows on the cost fields</t>
+  </si>
+  <si>
+    <t>1. Find a cost field with stepper arrows (small up/down buttons)
+2. Click the UP arrow once
+3. Observe how much the value increases
+4. Click the DOWN arrow once
+5. Observe how much the value decreases</t>
+  </si>
+  <si>
+    <t>1. Each click of the UP arrow should increase the value
+2. Each click of the DOWN arrow should decrease the value
+3. The increment should be small (typically 0.01 or 1)
+4. The value should not go below 0 when clicking down
+5. Note the actual increment amount for the test result</t>
+  </si>
+  <si>
+    <t>Add a new state to the resource</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Click the calendar/list icon (third tab) to open States
+3. The States editor is now visible
+4. You can see a list of existing states (or an empty list)</t>
+  </si>
+  <si>
+    <t>1. Look for an "Add" button or "+" icon in the States panel
+2. Click the "Add" button to create a new state
+3. A new state entry should appear in the list
+4. The new state may have a default name like "New State" or "State 1"</t>
+  </si>
+  <si>
+    <t>1. A new state row appears in the States list
+2. The new state has a default name that you can edit
+3. IMPORTANT: The change saves AUTOMATICALLY
+4. There is NO Save button to click - changes are instant
+5. You can now customize the new state's properties</t>
+  </si>
+  <si>
+    <t>Edit an existing state name</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. States tab is open (calendar/list icon selected)
+3. At least one state exists in the list
+4. You can see the state's name field</t>
+  </si>
+  <si>
+    <t>1. Find an existing state in the list
+2. Click on the state's name field (it may be a text box or editable label)
+3. Select the existing name text
+4. Type a new name like "Working" or "Busy"
+5. Press Tab or click outside the name field</t>
+  </si>
+  <si>
+    <t>1. The state's name changes to your new text (e.g., "Working")
+2. IMPORTANT: The change saves AUTOMATICALLY
+3. There is NO Save button needed
+4. The state list now shows the updated name
+5. This state name will appear in simulation reports</t>
+  </si>
+  <si>
+    <t>Delete an existing state</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. States tab is open (calendar/list icon selected)
+3. At least one state exists that you want to delete
+4. You can see the list of states</t>
+  </si>
+  <si>
+    <t>1. Find the state you want to delete in the list
+2. Look for a delete button (trash can icon, "×", or "Remove")
+   - It may appear when you hover over the state row
+   - Or it may be at the end of the state row
+3. Click the delete button
+4. Confirm deletion if prompted</t>
+  </si>
+  <si>
+    <t>1. The state is removed from the list
+2. IMPORTANT: The deletion saves AUTOMATICALLY
+3. There is NO Save button needed - the state is gone immediately
+4. The States list now has one fewer entry
+5. WARNING: This action may not be undoable</t>
+  </si>
+  <si>
+    <t>Verify States tab auto-saves changes</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. States tab is open (calendar/list icon selected)
+3. You have NOT made any changes yet</t>
+  </si>
+  <si>
+    <t>1. Make a change to the States (add, edit name, or delete)
+2. Immediately after, switch to a different tab (click gear icon)
+3. Then switch back to States tab (click calendar/list icon)
+4. Look at the States list</t>
+  </si>
+  <si>
+    <t>1. Your previous change is still there (persisted)
+2. This confirms auto-save is working
+3. Unlike Basic/Financial tabs, States does NOT require clicking Save
+4. All changes are saved immediately as you make them
+5. There is no "unsaved changes" state on this tab</t>
+  </si>
+  <si>
+    <t>Verify Save/Cancel buttons are hidden on States tab</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. States tab is open (calendar/list icon selected)
+3. You can see the States editor content</t>
+  </si>
+  <si>
+    <t>1. Look at the BOTTOM of the Resource Editor panel
+2. Look for any Save or Cancel buttons
+3. Compare to what you see on the Basic Settings tab
+4. Note whether these buttons are visible or hidden</t>
+  </si>
+  <si>
+    <t>1. The Save and Cancel buttons should NOT be visible
+2. The bottom of the panel should be empty or show different content
+3. This is because States auto-saves - no manual save is needed
+4. If you switch to Basic Settings tab, Save/Cancel buttons appear
+5. States tab behavior is different from other tabs</t>
+  </si>
+  <si>
+    <t>Save button initially disabled when no changes</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Click on a Resource shape (hexagon) in your diagram
+3. The Resource Editor panel appears on the right
+4. Click the gear icon to open Basic Settings tab
+5. You have NOT made any changes yet</t>
+  </si>
+  <si>
+    <t>1. Look at the BOTTOM of the Resource Editor panel
+2. Find the Save button (usually on the right side)
+3. Observe the button's appearance
+4. Try to click the Save button</t>
+  </si>
+  <si>
+    <t>1. The Save button should appear GRAYED OUT or dimmed
+2. The button should NOT be clickable
+3. Clicking it does nothing
+4. This is correct - there are no changes to save
+5. The button will become active only after you make a change</t>
+  </si>
+  <si>
+    <t>Save button enables when changes are made</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings or Financial Settings tab is open
+3. The Save button at the bottom is currently GRAYED OUT
+4. You have not made any changes yet</t>
+  </si>
+  <si>
+    <t>1. Make a change to any field:
+   - Change the Resource Name, OR
+   - Change the Capacity value, OR
+   - Toggle Financial Tracking, OR
+   - Change a cost value
+2. Look at the Save button immediately after making the change</t>
+  </si>
+  <si>
+    <t>1. The Save button changes from grayed out to BLUE (active)
+2. The button is now clickable
+3. This indicates there are unsaved changes
+4. The Cancel button should also be visible/active
+5. The form is now in a "dirty" state with pending changes</t>
+  </si>
+  <si>
+    <t>Save button persists changes</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings tab is open
+3. You have made a change (e.g., renamed the resource)
+4. The Save button is BLUE and clickable</t>
+  </si>
+  <si>
+    <t>1. Note the current value you changed (e.g., new name "Test Resource")
+2. Click the Save button
+3. Wait for the save to complete
+4. Switch to a different shape, then back to this Resource
+5. Check if your change is still there</t>
+  </si>
+  <si>
+    <t>1. After clicking Save, the button becomes grayed out again
+2. When you return to this Resource, your change is preserved
+3. The name (or other field) still shows your saved value
+4. This confirms the change was saved to the model
+5. The change persists even after switching elements</t>
+  </si>
+  <si>
+    <t>Cancel button discards changes</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings tab is open
+3. Note the ORIGINAL value of the Resource Name (e.g., "Resource 1")
+4. You have made a change but NOT saved yet</t>
+  </si>
+  <si>
+    <t>1. Change the Resource Name to something different (e.g., "Changed Name")
+2. Verify the Save button is now BLUE (active)
+3. Find the Cancel button (usually next to Save, or gray button)
+4. Click the Cancel button
+5. Look at the Resource Name field</t>
+  </si>
+  <si>
+    <t>1. The Resource Name field reverts to the ORIGINAL value ("Resource 1")
+2. Your change ("Changed Name") is DISCARDED
+3. The Save button becomes grayed out again
+4. The form returns to its clean state
+5. No changes were saved - the resource is unchanged</t>
+  </si>
+  <si>
+    <t>Changes persist when switching tabs (dirty state)</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings tab is open
+3. You have NOT made any changes yet</t>
+  </si>
+  <si>
+    <t>1. Change the Resource Name to "Tab Test"
+2. Verify the Save button is BLUE (active)
+3. Click the Financial Settings tab (dollar icon)
+4. Then click back to Basic Settings tab (gear icon)
+5. Look at the Resource Name field</t>
+  </si>
+  <si>
+    <t>1. The Resource Name still shows "Tab Test"
+2. Your unsaved change was NOT lost when switching tabs
+3. The Save button is still BLUE (active)
+4. The form remembers your pending changes
+5. You can continue editing or save/cancel</t>
+  </si>
+  <si>
+    <t>Save button shows loading state during save</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings tab is open
+3. You have made a change
+4. The Save button is BLUE and clickable</t>
+  </si>
+  <si>
+    <t>1. Click the Save button
+2. Watch the button IMMEDIATELY as you click
+3. Look for any text change or loading indicator
+4. This may happen quickly, so pay close attention</t>
+  </si>
+  <si>
+    <t>1. The Save button should briefly show "Saving..." text
+2. OR the button may show a loading spinner
+3. This loading state indicates the save is in progress
+4. After saving completes, the button returns to grayed out
+5. Note: This may happen very fast on local operations</t>
+  </si>
+  <si>
+    <t>Rapid Save button clicks handled correctly</t>
+  </si>
+  <si>
+    <t>1. Click the Save button rapidly 3-4 times in quick succession
+2. Watch what happens to the button and the form
+3. Check if any errors occur
+4. After the operation completes, verify the resource was saved correctly</t>
+  </si>
+  <si>
+    <t>1. Only ONE save operation should occur (not multiple)
+2. The application should NOT crash or freeze
+3. No error messages should appear
+4. The form should end up in a clean state (Save grayed out)
+5. The resource should be saved correctly</t>
+  </si>
+  <si>
+    <t>Cancel button after successful save does nothing</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings tab is open
+3. You have just successfully saved changes
+4. The Save button is now grayed out (no pending changes)</t>
+  </si>
+  <si>
+    <t>1. After saving, locate the Cancel button
+2. Click the Cancel button
+3. Observe what happens to the form
+4. Check if any values change</t>
+  </si>
+  <si>
+    <t>1. Nothing should change - there are no changes to cancel
+2. The form values remain the same as the saved values
+3. No error messages should appear
+4. The Cancel button may be grayed out (disabled)
+5. OR clicking it simply does nothing</t>
+  </si>
+  <si>
+    <t>Form loads data when switching to different resource</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Your model has at least 2 Resource shapes (hexagons)
+3. One resource is named "Resource A" and another "Resource B"
+4. Click on "Resource A" to select it
+5. The Resource Editor shows Resource A's data</t>
+  </si>
+  <si>
+    <t>1. Look at the current Resource Name displayed (should be "Resource A")
+2. In the DIAGRAM (not the panel), click on "Resource B" shape
+3. Watch the Resource Editor panel on the right
+4. Observe how the panel content changes</t>
+  </si>
+  <si>
+    <t>1. The panel title may change to show "Resource B" or indicate the new selection
+2. The Resource Name field now shows "Resource B" (not "Resource A")
+3. All other fields (Capacity, etc.) show Resource B's values
+4. The form completely refreshes to show the newly selected resource
+5. This happens automatically when you select a different shape</t>
+  </si>
+  <si>
+    <t>Unsaved changes are discarded when switching resources</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Your model has at least 2 Resource shapes
+3. Click on "Resource A" to select it
+4. The Resource Editor shows Resource A's data</t>
+  </si>
+  <si>
+    <t>1. Change Resource A's name to "Modified A" (do NOT click Save)
+2. Verify the Save button is BLUE (active)
+3. In the DIAGRAM, click on "Resource B" shape
+4. The panel now shows Resource B's data
+5. Now click back on "Resource A" in the diagram</t>
+  </si>
+  <si>
+    <t>1. When you switch to Resource B, the unsaved change is DISCARDED
+2. When you switch back to Resource A:
+   - The name shows the ORIGINAL name (NOT "Modified A")
+   - Your unsaved change was lost
+3. This is expected behavior - switching resources without saving loses changes
+4. IMPORTANT: Always Save before switching if you want to keep changes</t>
+  </si>
+  <si>
+    <t>External/collaborative updates sync to form</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Have a Resource shape selected in your diagram
+3. The Resource Editor shows the current resource data
+4. Another user has edit access to this document (collaborative editing)</t>
+  </si>
+  <si>
+    <t>1. Have another user (or another browser tab) open the same document
+2. In the OTHER session, change the Resource Name and Save
+3. In YOUR session, observe the Resource Editor panel
+4. You may need to re-select the resource to see updates</t>
+  </si>
+  <si>
+    <t>1. The form should eventually reflect the other user's changes
+2. This may happen:
+   - Automatically after a brief delay
+   - When you re-select the resource
+   - After the document syncs
+3. The Resource Name should show the new value from the other session
+4. This confirms collaborative editing works for resources
+5. Note: Real-time sync timing may vary</t>
+  </si>
+  <si>
+    <t>Editor handles resource with missing/corrupt data</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. The model may have a Resource with incomplete or corrupt data
+   (This can happen if the model was partially saved or imported incorrectly)
+3. Attempt to select this problematic Resource shape</t>
+  </si>
+  <si>
+    <t>1. Click on a Resource shape in the diagram
+2. If the resource has corrupt or missing required properties:
+   - Watch how the Resource Editor responds
+   - Look for any error messages
+3. Check if the panel displays something or shows an error</t>
+  </si>
+  <si>
+    <t>1. The editor should handle the error GRACEFULLY
+2. Either:
+   - Display an error message explaining the problem
+   - Show the editor with default/fallback values
+   - Indicate which fields are missing or invalid
+3. The application should NOT crash or freeze
+4. The user should understand what went wrong</t>
+  </si>
+  <si>
+    <t>Browser refresh with unsaved changes loses data</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Click on a Resource shape to select it
+3. The Resource Editor is open and showing the resource data</t>
+  </si>
+  <si>
+    <t>1. Change the Resource Name to "Unsaved Test"
+2. Verify the Save button is BLUE (active) - meaning you have unsaved changes
+3. WITHOUT clicking Save, refresh the browser:
+   - Press F5, or
+   - Press Ctrl+R, or
+   - Click the browser's refresh button
+4. Wait for the page to reload
+5. Select the same Resource again</t>
+  </si>
+  <si>
+    <t>1. Your unsaved change ("Unsaved Test") is LOST
+2. The Resource Name shows the ORIGINAL value (before your change)
+3. This is EXPECTED behavior - browser refresh loses unsaved work
+4. This test confirms that changes must be saved before refresh
+5. WARNING: There may be no warning prompt before refresh</t>
+  </si>
+  <si>
+    <t>Very high capacity value handling</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings tab is open (gear icon selected)
+3. You can see the Capacity field</t>
+  </si>
+  <si>
+    <t>1. Click inside the Capacity field
+2. Clear the current value
+3. Type a very large number: "999999"
+4. Press Tab or click outside the field
+5. Try to save the change</t>
+  </si>
+  <si>
+    <t>1. The Capacity field should accept the large value
+2. The field displays "999999" (or possibly formatted with commas)
+3. The application should NOT crash or freeze
+4. The Save button should become enabled
+5. You should be able to save successfully
+6. Note: Very high capacity may affect simulation performance</t>
+  </si>
+  <si>
+    <t>Non-numeric input in Capacity field</t>
+  </si>
+  <si>
+    <t>1. Have a Resource shape selected in your diagram
+2. Basic Settings tab is open (gear icon selected)
+3. You can see the Capacity field showing a number</t>
+  </si>
+  <si>
+    <t>1. Click inside the Capacity field
+2. Clear the current value
+3. Type non-numeric text: "abc"
+4. Press Tab or click outside the field
+5. Observe what happens to the field value</t>
+  </si>
+  <si>
+    <t>1. The Capacity field should REJECT non-numeric input
+2. Possible behaviors:
+   - The field reverts to 1 (minimum valid value)
+   - The field shows the previous valid value
+   - An error message appears
+   - The non-numeric characters are blocked from being typed
+3. The field should end up with a valid numeric value
+4. Note the actual behavior for the test result</t>
+  </si>
+  <si>
+    <t>Non-numeric input in cost fields</t>
+  </si>
+  <si>
+    <t>1. Click inside any cost field (e.g., Cost Per Seize)
+2. Clear the current value
+3. Type non-numeric text: "abc"
+4. Press Tab or click outside the field
+5. Observe what happens to the field value</t>
+  </si>
+  <si>
+    <t>1. The cost field should REJECT non-numeric input
+2. Possible behaviors:
+   - The field reverts to 0 (minimum valid value)
+   - The field shows the previous valid value
+   - An error message appears
+   - The non-numeric characters are blocked from being typed
+3. The field should end up with a valid numeric value
+4. Note the actual behavior for the test result</t>
+  </si>
+  <si>
+    <t>Missing resource name shows validation error</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Click on a Resource shape (hexagon) in your diagram
+3. The Resource Editor is open showing Basic Settings
+4. The Resource currently has a name</t>
+  </si>
+  <si>
+    <t>1. Clear the Resource Name field completely (leave it blank)
+2. Click the Save button to save the empty name
+3. Click on the Model icon in the diagram (or use Model Panel)
+4. Open the Validation tab in the Model Panel
+5. Look for errors related to this resource</t>
+  </si>
+  <si>
+    <t>1. The Validation tab shows an ERROR message
+2. The error indicates the resource has a missing or blank name
+3. Error text may say: "Missing name" or "Resource name required"
+4. The error should identify which resource has the problem
+5. This helps users find and fix incomplete resources</t>
+  </si>
+  <si>
+    <t>Invalid capacity (zero/negative) shows validation error</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Click on a Resource shape in your diagram
+3. The Resource Editor is open showing Basic Settings
+4. The Capacity field shows a valid number (e.g., 1)</t>
+  </si>
+  <si>
+    <t>1. Change the Capacity field to 0 (if allowed) or -1
+2. Save the resource if possible
+3. Open the Model Panel by clicking the Model icon
+4. Navigate to the Validation tab
+5. Look for errors related to resource capacity</t>
+  </si>
+  <si>
+    <t>1. The Validation tab shows an ERROR message about capacity
+2. Error text may say: "Invalid capacity" or "Capacity must be positive"
+3. The error identifies which resource has the invalid capacity
+4. Resources must have capacity &gt;= 1 to be useful
+5. The simulation cannot run with invalid capacity values</t>
+  </si>
+  <si>
+    <t>Non-integer capacity shows validation error</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Click on a Resource shape in your diagram
+3. The Resource Editor is open showing Basic Settings
+4. The Capacity field shows a whole number</t>
+  </si>
+  <si>
+    <t>1. Try to set the Capacity to a decimal value like "2.5"
+   (Note: The field may prevent this or round the value)
+2. If decimal is accepted, save the resource
+3. Open the Model Panel Validation tab
+4. Look for errors about non-integer capacity</t>
+  </si>
+  <si>
+    <t>1. If decimal capacity is accepted:
+   - Validation shows ERROR: "Capacity must be a whole number"
+2. If decimal capacity is prevented:
+   - The field may auto-round to nearest integer
+   - Or block decimal input entirely
+3. Resource capacity represents discrete units (people, machines)
+4. Fractional capacity doesn't make sense in simulation</t>
+  </si>
+  <si>
+    <t>Very high capacity shows validation warning</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Click on a Resource shape in your diagram
+3. The Resource Editor is open showing Basic Settings</t>
+  </si>
+  <si>
+    <t>1. Set the Capacity field to a very high value: 1000001 (over 1 million)
+2. Save the resource
+3. Open the Model Panel Validation tab
+4. Look for any warnings about this resource</t>
+  </si>
+  <si>
+    <t>1. The Validation tab may show a WARNING (not error)
+2. Warning text: "Unusually high capacity" or similar
+3. This is a WARNING, not an ERROR - the simulation can still run
+4. The warning alerts users to potentially unintended values
+5. Note: Some applications may accept large values without warning</t>
+  </si>
+  <si>
+    <t>Unused resource shows validation warning</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Create a new Resource shape (or use an existing one)
+3. Make sure this Resource is NOT used by any Activity
+   (No Activity has a Resource Requirement referencing it)</t>
+  </si>
+  <si>
+    <t>1. Ensure the Resource exists but no Activity uses it
+2. Open the Model Panel by clicking the Model icon
+3. Navigate to the Validation tab
+4. Look for warnings about unused resources</t>
+  </si>
+  <si>
+    <t>1. The Validation tab shows a WARNING message
+2. Warning text: "Resource not used by any activity" or similar
+3. This is a WARNING, not an ERROR - simulation can run
+4. The warning alerts users that the resource has no purpose
+5. Users should either add requirements or remove the resource</t>
+  </si>
+  <si>
+    <t>Invalid resource requirement reference shows error</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. An Activity has a Resource Requirement configured
+3. The requirement points to a specific Resource
+4. You have access to modify the Activity's requirements</t>
+  </si>
+  <si>
+    <t>1. Open the Activity that has a resource requirement
+2. Navigate to the Resource Requirements (Actions tab)
+3. Delete or modify the requirement so it references an invalid resource
+4. Save the Activity
+5. Open Model Panel Validation tab</t>
+  </si>
+  <si>
+    <t>1. The Validation tab shows an ERROR message
+2. Error text: "Invalid resource requirement reference" or similar
+3. The error identifies which Activity has the problem
+4. This can happen if a Resource Requirement becomes orphaned
+5. The Activity cannot seize a non-existent resource</t>
+  </si>
+  <si>
+    <t>Invalid resource quantity (zero/negative) shows error</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. An Activity has a Seize Resource action configured
+3. The action specifies a quantity of resources to seize</t>
+  </si>
+  <si>
+    <t>1. Open an Activity that has a Resource Requirement
+2. Find the Quantity field for the resource seize action
+3. Set the Quantity to 0 or a negative number
+4. Save the Activity
+5. Open Model Panel Validation tab</t>
+  </si>
+  <si>
+    <t>1. The Validation tab shows an ERROR message
+2. Error text: "Invalid resource quantity" or similar
+3. The quantity must be at least 1 to be meaningful
+4. You can't seize 0 or negative resources
+5. Fix by setting quantity to 1 or higher</t>
+  </si>
+  <si>
+    <t>Reference to deleted resource shows error</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. An Activity has a Resource Requirement referencing a Resource
+3. You are about to delete the Resource that is referenced</t>
+  </si>
+  <si>
+    <t>1. Note which Activity references the Resource
+2. Delete the Resource shape from the diagram
+3. Open the Model Panel by clicking the Model icon
+4. Navigate to the Validation tab
+5. Look for errors about missing resource references</t>
+  </si>
+  <si>
+    <t>1. The Validation tab shows an ERROR message
+2. Error text: "References non-existent resource" or similar
+3. The Activity still has a requirement but the Resource is gone
+4. The simulation cannot run with missing resource references
+5. Fix by: removing the requirement OR re-creating the Resource</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Create a Resource with Capacity = 1
+3. Create multiple Activities that all want to seize this Resource
+   (e.g., 3 Activities each requesting the same Resource)</t>
+  </si>
+  <si>
+    <t>1. Ensure the Resource has Capacity = 1
+2. Configure 2 or more Activities to seize this Resource
+3. Save all configurations
+4. Open the Model Panel Validation tab
+5. Look for warnings about resource utilization</t>
+  </si>
+  <si>
+    <t>1. The Validation tab may show a WARNING about overutilization
+2. Warning text: "Resource might be overutilized" or similar
+3. This means demand may exceed supply
+4. The simulation can still run - entities will queue/wait
+5. This is informational to help with model design</t>
+  </si>
+  <si>
+    <t>Fixing validation issue clears the error</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. A Resource has a validation ERROR (e.g., missing name)
+3. The error is visible in the Model Panel Validation tab</t>
+  </si>
+  <si>
+    <t>1. Note the current validation error for a Resource
+2. Click on that Resource in the diagram to select it
+3. FIX the issue (e.g., enter a name for the Resource)
+4. Save the Resource
+5. Return to the Model Panel Validation tab
+6. Look for the error you just fixed</t>
+  </si>
+  <si>
+    <t>1. The validation error should DISAPPEAR from the list
+2. If there were multiple errors, only the fixed one disappears
+3. The model validation updates after you save changes
+4. This confirms the fix was successful
+5. Repeat for other errors until validation passes</t>
+  </si>
+  <si>
+    <t>Multiple validation errors shown separately</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Create or modify a Resource to have MULTIPLE problems
+   (e.g., empty name AND invalid capacity)</t>
+  </si>
+  <si>
+    <t>1. Create a Resource with:
+   - Empty/blank name
+   - Invalid capacity (if possible, or another issue)
+2. Save the Resource
+3. Open the Model Panel Validation tab
+4. Count how many errors appear for this Resource</t>
+  </si>
+  <si>
+    <t>1. Each validation issue should be listed SEPARATELY
+2. For example:
+   - Error 1: "Missing name" for the Resource
+   - Error 2: "Invalid capacity" for the Resource
+3. Each error has its own row/entry in the validation list
+4. This helps users identify ALL issues, not just the first one
+5. Users can fix issues one by one</t>
+  </si>
+  <si>
+    <t>Clicking validation error navigates to the element</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. A Resource has a validation error showing in the Model Panel
+3. The Validation tab shows at least one error</t>
+  </si>
+  <si>
+    <t>1. Open the Model Panel Validation tab
+2. Find an error related to a Resource
+3. Click on the error item (the row or the resource name)
+4. Watch what happens in the diagram and panel</t>
+  </si>
+  <si>
+    <t>1. Clicking the error should navigate to/select that Resource
+2. The Resource shape may become highlighted or selected in the diagram
+3. The Resource Editor may open showing that Resource
+4. This makes it easy to find and fix the problematic element
+5. You don't have to hunt through the diagram manually</t>
+  </si>
+  <si>
+    <t>1. Have a LucidChart document open with a Quodsi model
+2. Create a Resource with Capacity = 2
+3. Configure 3 different Activities to each seize 1 of this Resource
+   (Total demand = 3, but capacity = 2)</t>
+  </si>
+  <si>
+    <t>1. Create Resource with Capacity = 2
+2. Create Activity 1: seize 1 of the Resource
+3. Create Activity 2: seize 1 of the Resource
+4. Create Activity 3: seize 1 of the Resource
+5. Save all configurations
+6. Open Model Panel Validation tab</t>
+  </si>
+  <si>
+    <t>1. Validation may show a WARNING about potential overutilization
+2. Warning: "Resource capacity (2) may be insufficient for demand (3)"
+3. This is advanced analysis comparing capacity to potential demand
+4. Note: This warning may not appear in all implementations
+5. If present, it helps users design better models
+6. The simulation will still run - entities will wait in queue</t>
   </si>
 </sst>
 </file>
@@ -937,9 +2197,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="false">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="false">
       <alignment/>
     </xf>
   </cellXfs>
@@ -1245,68 +2508,68 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col bestFit="true" customWidth="true" max="1" min="1" width="11.88671875"/>
+    <col bestFit="true" customWidth="true" max="2" min="2" width="6.88671875"/>
+    <col bestFit="true" customWidth="true" max="3" min="3" width="21.44140625"/>
+    <col bestFit="true" customWidth="true" max="4" min="4" width="15.88671875"/>
+    <col bestFit="true" customWidth="true" max="5" min="5" width="21.6640625"/>
+    <col bestFit="true" customWidth="true" max="6" min="6" width="28.88671875"/>
+    <col bestFit="true" customWidth="true" max="7" min="7" width="11.5546875"/>
+    <col bestFit="true" customWidth="true" max="8" min="8" width="6"/>
+    <col bestFit="true" customWidth="true" max="9" min="9" width="7.44140625"/>
+    <col bestFit="true" customWidth="true" max="11" min="11" width="10.77734375"/>
+    <col bestFit="true" customWidth="true" max="12" min="12" width="11.88671875"/>
+    <col bestFit="true" customWidth="true" max="13" min="13" width="5.88671875"/>
+    <col bestFit="true" customWidth="true" max="14" min="14" width="7.6640625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:14">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1314,19 +2577,19 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>283</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>284</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>285</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1334,19 +2597,19 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>287</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>288</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>289</v>
       </c>
       <c r="F3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -1357,16 +2620,16 @@
         <v>26</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>288</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
+        <v>291</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -1374,19 +2637,19 @@
         <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>293</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>294</v>
       </c>
       <c r="E5" t="s">
-        <v>31</v>
+        <v>295</v>
       </c>
       <c r="F5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -1394,16 +2657,16 @@
         <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>297</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>298</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>299</v>
       </c>
       <c r="F6" t="s">
-        <v>36</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -1414,68 +2677,68 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:N10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col bestFit="true" customWidth="true" max="1" min="1" width="13.21875"/>
+    <col bestFit="true" customWidth="true" max="2" min="2" width="6.88671875"/>
+    <col bestFit="true" customWidth="true" max="3" min="3" width="24"/>
+    <col bestFit="true" customWidth="true" max="4" min="4" width="12.88671875"/>
+    <col bestFit="true" customWidth="true" max="5" min="5" width="33.109375"/>
+    <col bestFit="true" customWidth="true" max="6" min="6" width="30.5546875"/>
+    <col bestFit="true" customWidth="true" max="7" min="7" width="11.5546875"/>
+    <col bestFit="true" customWidth="true" max="8" min="8" width="6"/>
+    <col bestFit="true" customWidth="true" max="9" min="9" width="7.44140625"/>
+    <col bestFit="true" customWidth="true" max="11" min="11" width="10.77734375"/>
+    <col bestFit="true" customWidth="true" max="12" min="12" width="11.88671875"/>
+    <col bestFit="true" customWidth="true" max="13" min="13" width="5.88671875"/>
+    <col bestFit="true" customWidth="true" max="14" min="14" width="7.6640625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:14">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -1486,16 +2749,16 @@
         <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>301</v>
       </c>
       <c r="E2" t="s">
-        <v>40</v>
+        <v>302</v>
       </c>
       <c r="F2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>42</v>
       </c>
@@ -1506,16 +2769,16 @@
         <v>43</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>304</v>
       </c>
       <c r="E3" t="s">
-        <v>44</v>
+        <v>305</v>
       </c>
       <c r="F3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>46</v>
       </c>
@@ -1523,19 +2786,19 @@
         <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>307</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>308</v>
       </c>
       <c r="E4" t="s">
-        <v>48</v>
+        <v>309</v>
       </c>
       <c r="F4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -1546,16 +2809,16 @@
         <v>51</v>
       </c>
       <c r="D5" t="s">
-        <v>39</v>
+        <v>311</v>
       </c>
       <c r="E5" t="s">
-        <v>52</v>
+        <v>312</v>
       </c>
       <c r="F5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>53</v>
       </c>
@@ -1566,16 +2829,16 @@
         <v>55</v>
       </c>
       <c r="D6" t="s">
-        <v>39</v>
+        <v>314</v>
       </c>
       <c r="E6" t="s">
-        <v>56</v>
+        <v>315</v>
       </c>
       <c r="F6" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
       <c r="A7" t="s">
         <v>58</v>
       </c>
@@ -1586,16 +2849,16 @@
         <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>317</v>
       </c>
       <c r="E7" t="s">
-        <v>60</v>
+        <v>318</v>
       </c>
       <c r="F7" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
       <c r="A8" t="s">
         <v>62</v>
       </c>
@@ -1603,19 +2866,19 @@
         <v>54</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>320</v>
       </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>317</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>321</v>
       </c>
       <c r="F8" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
       <c r="A9" t="s">
         <v>66</v>
       </c>
@@ -1623,19 +2886,19 @@
         <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>67</v>
+        <v>323</v>
       </c>
       <c r="D9" t="s">
-        <v>39</v>
+        <v>324</v>
       </c>
       <c r="E9" t="s">
-        <v>68</v>
+        <v>325</v>
       </c>
       <c r="F9" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
       <c r="A10" t="s">
         <v>70</v>
       </c>
@@ -1643,16 +2906,16 @@
         <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>71</v>
+        <v>327</v>
       </c>
       <c r="D10" t="s">
-        <v>39</v>
+        <v>328</v>
       </c>
       <c r="E10" t="s">
-        <v>72</v>
+        <v>329</v>
       </c>
       <c r="F10" t="s">
-        <v>73</v>
+        <v>330</v>
       </c>
     </row>
   </sheetData>
@@ -1663,68 +2926,68 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:N14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col bestFit="true" customWidth="true" max="1" min="1" width="11.109375"/>
+    <col bestFit="true" customWidth="true" max="2" min="2" width="6.88671875"/>
+    <col bestFit="true" customWidth="true" max="3" min="3" width="25"/>
+    <col bestFit="true" customWidth="true" max="4" min="4" width="15.88671875"/>
+    <col bestFit="true" customWidth="true" max="5" min="5" width="35.33203125"/>
+    <col bestFit="true" customWidth="true" max="6" min="6" width="30.5546875"/>
+    <col bestFit="true" customWidth="true" max="7" min="7" width="11.5546875"/>
+    <col bestFit="true" customWidth="true" max="8" min="8" width="6"/>
+    <col bestFit="true" customWidth="true" max="9" min="9" width="7.44140625"/>
+    <col bestFit="true" customWidth="true" max="11" min="11" width="10.77734375"/>
+    <col bestFit="true" customWidth="true" max="12" min="12" width="11.88671875"/>
+    <col bestFit="true" customWidth="true" max="13" min="13" width="5.88671875"/>
+    <col bestFit="true" customWidth="true" max="14" min="14" width="7.6640625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:14">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>74</v>
       </c>
@@ -1735,16 +2998,16 @@
         <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>76</v>
+        <v>331</v>
       </c>
       <c r="E2" t="s">
-        <v>77</v>
+        <v>332</v>
       </c>
       <c r="F2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>79</v>
       </c>
@@ -1755,16 +3018,16 @@
         <v>80</v>
       </c>
       <c r="D3" t="s">
-        <v>81</v>
+        <v>334</v>
       </c>
       <c r="E3" t="s">
-        <v>82</v>
+        <v>335</v>
       </c>
       <c r="F3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>84</v>
       </c>
@@ -1772,19 +3035,19 @@
         <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>85</v>
+        <v>337</v>
       </c>
       <c r="D4" t="s">
-        <v>81</v>
+        <v>338</v>
       </c>
       <c r="E4" t="s">
-        <v>86</v>
+        <v>339</v>
       </c>
       <c r="F4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>88</v>
       </c>
@@ -1792,19 +3055,19 @@
         <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>89</v>
+        <v>341</v>
       </c>
       <c r="D5" t="s">
-        <v>81</v>
+        <v>338</v>
       </c>
       <c r="E5" t="s">
-        <v>90</v>
+        <v>342</v>
       </c>
       <c r="F5" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>92</v>
       </c>
@@ -1812,19 +3075,19 @@
         <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>93</v>
+        <v>344</v>
       </c>
       <c r="D6" t="s">
-        <v>81</v>
+        <v>338</v>
       </c>
       <c r="E6" t="s">
-        <v>94</v>
+        <v>345</v>
       </c>
       <c r="F6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
       <c r="A7" t="s">
         <v>95</v>
       </c>
@@ -1832,19 +3095,19 @@
         <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>96</v>
+        <v>347</v>
       </c>
       <c r="D7" t="s">
-        <v>81</v>
+        <v>348</v>
       </c>
       <c r="E7" t="s">
-        <v>97</v>
+        <v>349</v>
       </c>
       <c r="F7" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
       <c r="A8" t="s">
         <v>99</v>
       </c>
@@ -1852,19 +3115,19 @@
         <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>351</v>
       </c>
       <c r="D8" t="s">
-        <v>81</v>
+        <v>338</v>
       </c>
       <c r="E8" t="s">
-        <v>101</v>
+        <v>352</v>
       </c>
       <c r="F8" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
       <c r="A9" t="s">
         <v>103</v>
       </c>
@@ -1872,19 +3135,19 @@
         <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>354</v>
       </c>
       <c r="D9" t="s">
-        <v>81</v>
+        <v>338</v>
       </c>
       <c r="E9" t="s">
-        <v>105</v>
+        <v>355</v>
       </c>
       <c r="F9" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
       <c r="A10" t="s">
         <v>107</v>
       </c>
@@ -1895,16 +3158,16 @@
         <v>108</v>
       </c>
       <c r="D10" t="s">
-        <v>81</v>
+        <v>338</v>
       </c>
       <c r="E10" t="s">
-        <v>109</v>
+        <v>357</v>
       </c>
       <c r="F10" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
       <c r="A11" t="s">
         <v>111</v>
       </c>
@@ -1912,19 +3175,19 @@
         <v>25</v>
       </c>
       <c r="C11" t="s">
-        <v>112</v>
+        <v>359</v>
       </c>
       <c r="D11" t="s">
-        <v>81</v>
+        <v>338</v>
       </c>
       <c r="E11" t="s">
-        <v>113</v>
+        <v>360</v>
       </c>
       <c r="F11" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
       <c r="A12" t="s">
         <v>115</v>
       </c>
@@ -1932,19 +3195,19 @@
         <v>25</v>
       </c>
       <c r="C12" t="s">
-        <v>116</v>
+        <v>362</v>
       </c>
       <c r="D12" t="s">
-        <v>81</v>
+        <v>338</v>
       </c>
       <c r="E12" t="s">
-        <v>117</v>
+        <v>363</v>
       </c>
       <c r="F12" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
       <c r="A13" t="s">
         <v>119</v>
       </c>
@@ -1952,19 +3215,19 @@
         <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>120</v>
+        <v>365</v>
       </c>
       <c r="D13" t="s">
-        <v>81</v>
+        <v>338</v>
       </c>
       <c r="E13" t="s">
-        <v>121</v>
+        <v>366</v>
       </c>
       <c r="F13" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
       <c r="A14" t="s">
         <v>123</v>
       </c>
@@ -1972,16 +3235,16 @@
         <v>54</v>
       </c>
       <c r="C14" t="s">
-        <v>124</v>
+        <v>368</v>
       </c>
       <c r="D14" t="s">
-        <v>81</v>
+        <v>369</v>
       </c>
       <c r="E14" t="s">
-        <v>125</v>
+        <v>370</v>
       </c>
       <c r="F14" t="s">
-        <v>126</v>
+        <v>371</v>
       </c>
     </row>
   </sheetData>
@@ -1992,68 +3255,68 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:N6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col bestFit="true" customWidth="true" max="1" min="1" width="13.44140625"/>
+    <col bestFit="true" customWidth="true" max="2" min="2" width="6.88671875"/>
+    <col bestFit="true" customWidth="true" max="3" min="3" width="24.88671875"/>
+    <col bestFit="true" customWidth="true" max="4" min="4" width="13.77734375"/>
+    <col bestFit="true" customWidth="true" max="5" min="5" width="25.88671875"/>
+    <col bestFit="true" customWidth="true" max="6" min="6" width="30.33203125"/>
+    <col bestFit="true" customWidth="true" max="7" min="7" width="11.5546875"/>
+    <col bestFit="true" customWidth="true" max="8" min="8" width="6"/>
+    <col bestFit="true" customWidth="true" max="9" min="9" width="7.44140625"/>
+    <col bestFit="true" customWidth="true" max="11" min="11" width="10.77734375"/>
+    <col bestFit="true" customWidth="true" max="12" min="12" width="11.88671875"/>
+    <col bestFit="true" customWidth="true" max="13" min="13" width="5.88671875"/>
+    <col bestFit="true" customWidth="true" max="14" min="14" width="7.6640625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:14">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>127</v>
       </c>
@@ -2061,19 +3324,19 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>128</v>
+        <v>372</v>
       </c>
       <c r="D2" t="s">
-        <v>129</v>
+        <v>373</v>
       </c>
       <c r="E2" t="s">
-        <v>130</v>
+        <v>374</v>
       </c>
       <c r="F2" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>132</v>
       </c>
@@ -2081,19 +3344,19 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>133</v>
+        <v>376</v>
       </c>
       <c r="D3" t="s">
-        <v>134</v>
+        <v>377</v>
       </c>
       <c r="E3" t="s">
-        <v>135</v>
+        <v>378</v>
       </c>
       <c r="F3" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>137</v>
       </c>
@@ -2101,19 +3364,19 @@
         <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>138</v>
+        <v>380</v>
       </c>
       <c r="D4" t="s">
-        <v>134</v>
+        <v>381</v>
       </c>
       <c r="E4" t="s">
-        <v>139</v>
+        <v>382</v>
       </c>
       <c r="F4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>141</v>
       </c>
@@ -2121,19 +3384,19 @@
         <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>142</v>
+        <v>384</v>
       </c>
       <c r="D5" t="s">
-        <v>129</v>
+        <v>385</v>
       </c>
       <c r="E5" t="s">
-        <v>143</v>
+        <v>386</v>
       </c>
       <c r="F5" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>145</v>
       </c>
@@ -2141,16 +3404,16 @@
         <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>146</v>
+        <v>388</v>
       </c>
       <c r="D6" t="s">
-        <v>129</v>
+        <v>389</v>
       </c>
       <c r="E6" t="s">
-        <v>147</v>
+        <v>390</v>
       </c>
       <c r="F6" t="s">
-        <v>148</v>
+        <v>391</v>
       </c>
     </row>
   </sheetData>
@@ -2161,68 +3424,68 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:N9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col bestFit="true" customWidth="true" max="1" min="1" width="12.44140625"/>
+    <col bestFit="true" customWidth="true" max="2" min="2" width="6.88671875"/>
+    <col bestFit="true" customWidth="true" max="3" min="3" width="26.5546875"/>
+    <col bestFit="true" customWidth="true" max="4" min="4" width="19.33203125"/>
+    <col bestFit="true" customWidth="true" max="5" min="5" width="28.109375"/>
+    <col bestFit="true" customWidth="true" max="6" min="6" width="30.88671875"/>
+    <col bestFit="true" customWidth="true" max="7" min="7" width="11.5546875"/>
+    <col bestFit="true" customWidth="true" max="8" min="8" width="6"/>
+    <col bestFit="true" customWidth="true" max="9" min="9" width="7.44140625"/>
+    <col bestFit="true" customWidth="true" max="11" min="11" width="10.77734375"/>
+    <col bestFit="true" customWidth="true" max="12" min="12" width="11.88671875"/>
+    <col bestFit="true" customWidth="true" max="13" min="13" width="5.88671875"/>
+    <col bestFit="true" customWidth="true" max="14" min="14" width="7.6640625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:14">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>149</v>
       </c>
@@ -2230,19 +3493,19 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>150</v>
+        <v>392</v>
       </c>
       <c r="D2" t="s">
-        <v>151</v>
+        <v>393</v>
       </c>
       <c r="E2" t="s">
-        <v>152</v>
+        <v>394</v>
       </c>
       <c r="F2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>154</v>
       </c>
@@ -2250,19 +3513,19 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>155</v>
+        <v>396</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>397</v>
       </c>
       <c r="E3" t="s">
-        <v>156</v>
+        <v>398</v>
       </c>
       <c r="F3" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>158</v>
       </c>
@@ -2270,19 +3533,19 @@
         <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>159</v>
+        <v>400</v>
       </c>
       <c r="D4" t="s">
-        <v>160</v>
+        <v>401</v>
       </c>
       <c r="E4" t="s">
-        <v>161</v>
+        <v>402</v>
       </c>
       <c r="F4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>163</v>
       </c>
@@ -2290,19 +3553,19 @@
         <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>164</v>
+        <v>404</v>
       </c>
       <c r="D5" t="s">
-        <v>160</v>
+        <v>405</v>
       </c>
       <c r="E5" t="s">
-        <v>165</v>
+        <v>406</v>
       </c>
       <c r="F5" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>167</v>
       </c>
@@ -2310,19 +3573,19 @@
         <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>168</v>
+        <v>408</v>
       </c>
       <c r="D6" t="s">
-        <v>160</v>
+        <v>409</v>
       </c>
       <c r="E6" t="s">
-        <v>169</v>
+        <v>410</v>
       </c>
       <c r="F6" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
       <c r="A7" t="s">
         <v>171</v>
       </c>
@@ -2330,19 +3593,19 @@
         <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>172</v>
+        <v>412</v>
       </c>
       <c r="D7" t="s">
-        <v>160</v>
+        <v>413</v>
       </c>
       <c r="E7" t="s">
-        <v>173</v>
+        <v>414</v>
       </c>
       <c r="F7" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
       <c r="A8" t="s">
         <v>175</v>
       </c>
@@ -2350,19 +3613,19 @@
         <v>54</v>
       </c>
       <c r="C8" t="s">
-        <v>176</v>
+        <v>416</v>
       </c>
       <c r="D8" t="s">
-        <v>160</v>
+        <v>413</v>
       </c>
       <c r="E8" t="s">
-        <v>177</v>
+        <v>417</v>
       </c>
       <c r="F8" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
       <c r="A9" t="s">
         <v>179</v>
       </c>
@@ -2370,16 +3633,16 @@
         <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>180</v>
+        <v>419</v>
       </c>
       <c r="D9" t="s">
-        <v>181</v>
+        <v>420</v>
       </c>
       <c r="E9" t="s">
-        <v>182</v>
+        <v>421</v>
       </c>
       <c r="F9" t="s">
-        <v>183</v>
+        <v>422</v>
       </c>
     </row>
   </sheetData>
@@ -2390,68 +3653,68 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:N4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="37.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col bestFit="true" customWidth="true" max="1" min="1" width="12.6640625"/>
+    <col bestFit="true" customWidth="true" max="2" min="2" width="6.88671875"/>
+    <col bestFit="true" customWidth="true" max="3" min="3" width="24.77734375"/>
+    <col bestFit="true" customWidth="true" max="4" min="4" width="21.88671875"/>
+    <col bestFit="true" customWidth="true" max="5" min="5" width="34"/>
+    <col bestFit="true" customWidth="true" max="6" min="6" width="37.88671875"/>
+    <col bestFit="true" customWidth="true" max="7" min="7" width="11.5546875"/>
+    <col bestFit="true" customWidth="true" max="8" min="8" width="6"/>
+    <col bestFit="true" customWidth="true" max="9" min="9" width="7.44140625"/>
+    <col bestFit="true" customWidth="true" max="11" min="11" width="10.77734375"/>
+    <col bestFit="true" customWidth="true" max="12" min="12" width="11.88671875"/>
+    <col bestFit="true" customWidth="true" max="13" min="13" width="5.88671875"/>
+    <col bestFit="true" customWidth="true" max="14" min="14" width="7.6640625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:14">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>184</v>
       </c>
@@ -2459,19 +3722,19 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>185</v>
+        <v>423</v>
       </c>
       <c r="D2" t="s">
-        <v>186</v>
+        <v>424</v>
       </c>
       <c r="E2" t="s">
-        <v>187</v>
+        <v>425</v>
       </c>
       <c r="F2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>189</v>
       </c>
@@ -2479,19 +3742,19 @@
         <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>190</v>
+        <v>427</v>
       </c>
       <c r="D3" t="s">
-        <v>191</v>
+        <v>428</v>
       </c>
       <c r="E3" t="s">
-        <v>192</v>
+        <v>429</v>
       </c>
       <c r="F3" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>194</v>
       </c>
@@ -2499,16 +3762,16 @@
         <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>195</v>
+        <v>431</v>
       </c>
       <c r="D4" t="s">
-        <v>196</v>
+        <v>432</v>
       </c>
       <c r="E4" t="s">
-        <v>197</v>
+        <v>433</v>
       </c>
       <c r="F4" t="s">
-        <v>198</v>
+        <v>434</v>
       </c>
     </row>
   </sheetData>
@@ -2519,68 +3782,68 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:N6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col bestFit="true" customWidth="true" max="1" min="1" width="12.77734375"/>
+    <col bestFit="true" customWidth="true" max="2" min="2" width="6.88671875"/>
+    <col bestFit="true" customWidth="true" max="3" min="3" width="23.77734375"/>
+    <col bestFit="true" customWidth="true" max="4" min="4" width="21.88671875"/>
+    <col bestFit="true" customWidth="true" max="5" min="5" width="33.88671875"/>
+    <col bestFit="true" customWidth="true" max="6" min="6" width="29.33203125"/>
+    <col bestFit="true" customWidth="true" max="7" min="7" width="11.5546875"/>
+    <col bestFit="true" customWidth="true" max="8" min="8" width="6"/>
+    <col bestFit="true" customWidth="true" max="9" min="9" width="7.44140625"/>
+    <col bestFit="true" customWidth="true" max="11" min="11" width="10.77734375"/>
+    <col bestFit="true" customWidth="true" max="12" min="12" width="11.88671875"/>
+    <col bestFit="true" customWidth="true" max="13" min="13" width="5.88671875"/>
+    <col bestFit="true" customWidth="true" max="14" min="14" width="7.6640625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:14">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>199</v>
       </c>
@@ -2588,19 +3851,19 @@
         <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>200</v>
+        <v>435</v>
       </c>
       <c r="D2" t="s">
-        <v>201</v>
+        <v>436</v>
       </c>
       <c r="E2" t="s">
-        <v>202</v>
+        <v>437</v>
       </c>
       <c r="F2" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>204</v>
       </c>
@@ -2608,19 +3871,19 @@
         <v>54</v>
       </c>
       <c r="C3" t="s">
-        <v>205</v>
+        <v>439</v>
       </c>
       <c r="D3" t="s">
-        <v>191</v>
+        <v>440</v>
       </c>
       <c r="E3" t="s">
-        <v>206</v>
+        <v>441</v>
       </c>
       <c r="F3" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>208</v>
       </c>
@@ -2628,19 +3891,19 @@
         <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>209</v>
+        <v>443</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>444</v>
       </c>
       <c r="E4" t="s">
-        <v>210</v>
+        <v>445</v>
       </c>
       <c r="F4" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>212</v>
       </c>
@@ -2648,19 +3911,19 @@
         <v>54</v>
       </c>
       <c r="C5" t="s">
-        <v>213</v>
+        <v>447</v>
       </c>
       <c r="D5" t="s">
-        <v>39</v>
+        <v>448</v>
       </c>
       <c r="E5" t="s">
-        <v>214</v>
+        <v>449</v>
       </c>
       <c r="F5" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>216</v>
       </c>
@@ -2668,16 +3931,16 @@
         <v>54</v>
       </c>
       <c r="C6" t="s">
-        <v>217</v>
+        <v>451</v>
       </c>
       <c r="D6" t="s">
-        <v>81</v>
+        <v>338</v>
       </c>
       <c r="E6" t="s">
-        <v>218</v>
+        <v>452</v>
       </c>
       <c r="F6" t="s">
-        <v>219</v>
+        <v>453</v>
       </c>
     </row>
   </sheetData>
@@ -2690,46 +3953,46 @@
   <dimension ref="A1:N14"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2741,16 +4004,16 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>221</v>
+        <v>454</v>
       </c>
       <c r="D2" t="s">
-        <v>222</v>
+        <v>455</v>
       </c>
       <c r="E2" t="s">
-        <v>223</v>
+        <v>456</v>
       </c>
       <c r="F2" t="s">
-        <v>224</v>
+        <v>457</v>
       </c>
       <c r="G2" t="s">
         <v>225</v>
@@ -2785,16 +4048,16 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>227</v>
+        <v>458</v>
       </c>
       <c r="D3" t="s">
-        <v>228</v>
+        <v>459</v>
       </c>
       <c r="E3" t="s">
-        <v>229</v>
+        <v>460</v>
       </c>
       <c r="F3" t="s">
-        <v>230</v>
+        <v>461</v>
       </c>
       <c r="G3" t="s">
         <v>225</v>
@@ -2829,16 +4092,16 @@
         <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>232</v>
+        <v>462</v>
       </c>
       <c r="D4" t="s">
-        <v>228</v>
+        <v>463</v>
       </c>
       <c r="E4" t="s">
-        <v>233</v>
+        <v>464</v>
       </c>
       <c r="F4" t="s">
-        <v>234</v>
+        <v>465</v>
       </c>
       <c r="G4" t="s">
         <v>225</v>
@@ -2873,16 +4136,16 @@
         <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>236</v>
+        <v>466</v>
       </c>
       <c r="D5" t="s">
-        <v>228</v>
+        <v>467</v>
       </c>
       <c r="E5" t="s">
-        <v>237</v>
+        <v>468</v>
       </c>
       <c r="F5" t="s">
-        <v>238</v>
+        <v>469</v>
       </c>
       <c r="G5" t="s">
         <v>225</v>
@@ -2917,16 +4180,16 @@
         <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>240</v>
+        <v>470</v>
       </c>
       <c r="D6" t="s">
-        <v>241</v>
+        <v>471</v>
       </c>
       <c r="E6" t="s">
-        <v>242</v>
+        <v>472</v>
       </c>
       <c r="F6" t="s">
-        <v>243</v>
+        <v>473</v>
       </c>
       <c r="G6" t="s">
         <v>225</v>
@@ -2961,16 +4224,16 @@
         <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>245</v>
+        <v>474</v>
       </c>
       <c r="D7" t="s">
-        <v>246</v>
+        <v>475</v>
       </c>
       <c r="E7" t="s">
-        <v>247</v>
+        <v>476</v>
       </c>
       <c r="F7" t="s">
-        <v>248</v>
+        <v>477</v>
       </c>
       <c r="G7" t="s">
         <v>225</v>
@@ -3005,16 +4268,16 @@
         <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>250</v>
+        <v>478</v>
       </c>
       <c r="D8" t="s">
-        <v>251</v>
+        <v>479</v>
       </c>
       <c r="E8" t="s">
-        <v>252</v>
+        <v>480</v>
       </c>
       <c r="F8" t="s">
-        <v>253</v>
+        <v>481</v>
       </c>
       <c r="G8" t="s">
         <v>225</v>
@@ -3049,16 +4312,16 @@
         <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>255</v>
+        <v>482</v>
       </c>
       <c r="D9" t="s">
-        <v>246</v>
+        <v>483</v>
       </c>
       <c r="E9" t="s">
-        <v>256</v>
+        <v>484</v>
       </c>
       <c r="F9" t="s">
-        <v>257</v>
+        <v>485</v>
       </c>
       <c r="G9" t="s">
         <v>225</v>
@@ -3096,13 +4359,13 @@
         <v>259</v>
       </c>
       <c r="D10" t="s">
-        <v>260</v>
+        <v>486</v>
       </c>
       <c r="E10" t="s">
-        <v>261</v>
+        <v>487</v>
       </c>
       <c r="F10" t="s">
-        <v>262</v>
+        <v>488</v>
       </c>
       <c r="G10" t="s">
         <v>225</v>
@@ -3137,16 +4400,16 @@
         <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>264</v>
+        <v>489</v>
       </c>
       <c r="D11" t="s">
-        <v>265</v>
+        <v>490</v>
       </c>
       <c r="E11" t="s">
-        <v>266</v>
+        <v>491</v>
       </c>
       <c r="F11" t="s">
-        <v>267</v>
+        <v>492</v>
       </c>
       <c r="G11" t="s">
         <v>225</v>
@@ -3181,16 +4444,16 @@
         <v>25</v>
       </c>
       <c r="C12" t="s">
-        <v>269</v>
+        <v>493</v>
       </c>
       <c r="D12" t="s">
-        <v>270</v>
+        <v>494</v>
       </c>
       <c r="E12" t="s">
-        <v>271</v>
+        <v>495</v>
       </c>
       <c r="F12" t="s">
-        <v>272</v>
+        <v>496</v>
       </c>
       <c r="G12" t="s">
         <v>225</v>
@@ -3225,16 +4488,16 @@
         <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>274</v>
+        <v>497</v>
       </c>
       <c r="D13" t="s">
-        <v>275</v>
+        <v>498</v>
       </c>
       <c r="E13" t="s">
-        <v>276</v>
+        <v>499</v>
       </c>
       <c r="F13" t="s">
-        <v>277</v>
+        <v>500</v>
       </c>
       <c r="G13" t="s">
         <v>225</v>
@@ -3272,13 +4535,13 @@
         <v>279</v>
       </c>
       <c r="D14" t="s">
-        <v>280</v>
+        <v>501</v>
       </c>
       <c r="E14" t="s">
-        <v>281</v>
+        <v>502</v>
       </c>
       <c r="F14" t="s">
-        <v>282</v>
+        <v>503</v>
       </c>
       <c r="G14" t="s">
         <v>225</v>

</xml_diff>